<commit_message>
next: do the columns
</commit_message>
<xml_diff>
--- a/calendar_config.xlsx
+++ b/calendar_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\coffee-salad-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE477495-03AA-4709-B02F-4715A1AA54D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B7669B9-B1A2-4A58-88D8-6E7C189AC975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11490" yWindow="3240" windowWidth="37305" windowHeight="15885" tabRatio="850" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9045" yWindow="1530" windowWidth="37305" windowHeight="15885" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="config-meta" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="264">
   <si>
     <t>param</t>
   </si>
@@ -357,30 +357,9 @@
     <t>annotation</t>
   </si>
   <si>
-    <t>iterate</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>does this column iterate</t>
-  </si>
-  <si>
-    <t>start</t>
-  </si>
-  <si>
     <t>int</t>
   </si>
   <si>
-    <t xml:space="preserve">start the increment on this </t>
-  </si>
-  <si>
-    <t>increment</t>
-  </si>
-  <si>
-    <t>incrementign value</t>
-  </si>
-  <si>
     <t>#terms</t>
   </si>
   <si>
@@ -495,9 +474,6 @@
     <t># week</t>
   </si>
   <si>
-    <t>iterator</t>
-  </si>
-  <si>
     <t>terms</t>
   </si>
   <si>
@@ -852,9 +828,6 @@
     <t>weekno_column</t>
   </si>
   <si>
-    <t>incrementing value</t>
-  </si>
-  <si>
     <t>semester 1</t>
   </si>
   <si>
@@ -864,7 +837,10 @@
     <t>semester 3</t>
   </si>
   <si>
-    <t>Now calculated using dates and the weekno_column</t>
+    <t># uni</t>
+  </si>
+  <si>
+    <t>Week number</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1312,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -1347,7 +1323,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1355,15 +1331,15 @@
         <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1371,15 +1347,15 @@
         <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B6" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1387,15 +1363,15 @@
         <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B8" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1403,7 +1379,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1411,7 +1387,7 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -1424,7 +1400,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1457,7 +1433,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1477,7 +1453,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1489,114 +1465,72 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>101</v>
+        <v>168</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1621,11 +1555,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1636,7 +1567,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1669,7 +1600,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1689,7 +1620,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1701,7 +1632,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -1712,106 +1643,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1836,11 +1725,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1851,7 +1737,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1884,7 +1770,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1904,7 +1790,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1916,7 +1802,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -1927,106 +1813,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2051,11 +1895,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2066,7 +1907,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -2099,7 +1940,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2119,7 +1960,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2131,7 +1972,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -2142,106 +1983,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2266,11 +2065,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2281,7 +2077,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -2314,7 +2110,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2334,7 +2130,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2346,7 +2142,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -2357,106 +2153,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2481,11 +2235,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2496,7 +2247,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -2529,7 +2280,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2549,7 +2300,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2561,7 +2312,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -2572,106 +2323,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2696,11 +2405,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2711,7 +2417,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -2744,7 +2450,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2764,7 +2470,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2776,7 +2482,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -2787,106 +2493,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2911,11 +2575,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2926,7 +2587,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -2959,7 +2620,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2979,7 +2640,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2991,7 +2652,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -3002,106 +2663,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3126,11 +2745,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3141,7 +2757,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -3174,7 +2790,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -3194,7 +2810,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3217,106 +2833,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3341,11 +2915,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3356,7 +2927,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -3432,106 +3003,64 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>105</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>111</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3556,11 +3085,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3603,7 +3129,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -3625,7 +3151,7 @@
     </row>
     <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -3635,41 +3161,41 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D8" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="B9" t="s">
         <v>70</v>
@@ -3678,12 +3204,12 @@
         <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
@@ -3692,24 +3218,24 @@
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="F10" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="B11" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C11" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="D11" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -5367,7 +4893,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -5382,111 +4908,111 @@
     <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D7" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B8" t="s">
         <v>100</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D8" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C9" s="14">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="E9" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C10" s="14">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E10" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="C11" s="15">
         <v>45658</v>
       </c>
       <c r="D11" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="C12" s="15">
         <v>46022</v>
       </c>
       <c r="D12" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C13" s="14">
         <v>1</v>
@@ -5494,10 +5020,10 @@
     </row>
     <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C14" s="14">
         <v>1</v>
@@ -5505,84 +5031,84 @@
     </row>
     <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C15" s="14">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="E15" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="B16" t="s">
         <v>100</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="D16" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E16" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B19" t="s">
         <v>100</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="D19" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="B20" t="s">
         <v>100</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D20" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="B21" t="s">
         <v>100</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="D21" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -5738,7 +5264,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -5753,60 +5279,60 @@
     <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D5" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="B6" t="s">
         <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="B7" t="s">
         <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="E10" s="7"/>
     </row>
@@ -5815,26 +5341,26 @@
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B13" t="s">
         <v>70</v>
       </c>
       <c r="C13" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="E13" s="7"/>
     </row>
     <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5845,171 +5371,171 @@
         <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B19" t="s">
         <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B22" t="s">
         <v>70</v>
       </c>
       <c r="C22" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="B25" t="s">
         <v>70</v>
       </c>
       <c r="C25" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B28" t="s">
         <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="B31" t="s">
         <v>70</v>
       </c>
       <c r="C31" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s">
         <v>70</v>
       </c>
       <c r="C34" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B37" t="s">
         <v>70</v>
       </c>
       <c r="C37" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B40" t="s">
         <v>70</v>
       </c>
       <c r="C40" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B43" t="s">
         <v>70</v>
       </c>
       <c r="C43" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="45" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B46" t="s">
         <v>70</v>
@@ -6021,7 +5547,7 @@
     <row r="47" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G48" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -6034,7 +5560,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -6067,7 +5593,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -6087,7 +5613,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6098,103 +5624,225 @@
       <c r="B7" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>148</v>
+      <c r="C7" t="s">
+        <v>158</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
       </c>
+      <c r="E7" s="7" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E8" s="11"/>
+    </row>
+    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="11"/>
+    </row>
+    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="14">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="11"/>
+    </row>
+    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" s="11"/>
+    </row>
+    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:F42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" t="s">
+        <v>55</v>
+      </c>
       <c r="E7" s="7"/>
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>271</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="11"/>
+    </row>
+    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="14">
-        <v>1</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
-      </c>
-      <c r="E10" s="11"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>107</v>
+      </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>165</v>
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
       </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" s="14">
-        <v>6</v>
-      </c>
-      <c r="D13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="D14" t="s">
-        <v>116</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E15" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6220,220 +5868,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:F45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E9" s="11"/>
-    </row>
-    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>1</v>
-      </c>
-      <c r="D10" t="s">
-        <v>267</v>
-      </c>
-      <c r="E10" s="11"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>149</v>
-      </c>
-      <c r="B11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6466,10 +5902,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>62</v>
@@ -6486,13 +5922,13 @@
     </row>
     <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
@@ -6506,103 +5942,103 @@
     </row>
     <row r="5" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C5" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D7" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E7" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F7" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F8" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="D9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F9" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D10" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E10" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F10" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="H10" s="11"/>
     </row>
@@ -6663,7 +6099,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -6696,7 +6132,7 @@
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -6716,7 +6152,7 @@
     </row>
     <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6728,7 +6164,7 @@
         <v>100</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>148</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
         <v>55</v>
@@ -6737,103 +6173,61 @@
     </row>
     <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>70</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="14">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>107</v>
-      </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>149</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>150</v>
+        <v>102</v>
+      </c>
+      <c r="C11" s="14">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>107</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="7"/>
-    </row>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6858,11 +6252,8 @@
     <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6895,10 +6286,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>62</v>
@@ -6909,13 +6300,13 @@
     </row>
     <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6926,103 +6317,103 @@
     </row>
     <row r="5" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D5" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="E5" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E7" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F7" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F8" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F9" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F10" t="s">
         <v>139</v>
-      </c>
-      <c r="E10" t="s">
-        <v>139</v>
-      </c>
-      <c r="F10" t="s">
-        <v>146</v>
       </c>
       <c r="H10" s="11"/>
     </row>

</xml_diff>